<commit_message>
Complete system overhaul with dynamic avatars and UI fixes
</commit_message>
<xml_diff>
--- a/islami-assistant-web/public/data/الفروع.xlsx
+++ b/islami-assistant-web/public/data/الفروع.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BLACK-DIAMOND\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BLACK-DIAMOND\Desktop\islami Assistant\islami-assistant-web\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BC6BF83-6B07-4D75-B448-1406158BF2E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D39B4C3-F737-4BA9-9127-4AD497525435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -342,7 +342,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="عادي" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -643,7 +643,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="31.5">
+    <row r="2" spans="1:4" ht="15.75">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -657,7 +657,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="47.25">
+    <row r="3" spans="1:4" ht="15.75">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -671,7 +671,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="31.5">
+    <row r="4" spans="1:4" ht="15.75">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -685,7 +685,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="31.5">
+    <row r="5" spans="1:4" ht="15.75">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
@@ -697,7 +697,7 @@
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:4" ht="31.5">
+    <row r="6" spans="1:4" ht="15.75">
       <c r="A6" s="1" t="s">
         <v>19</v>
       </c>
@@ -711,7 +711,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="47.25">
+    <row r="7" spans="1:4" ht="15.75">
       <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
@@ -725,7 +725,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="31.5">
+    <row r="8" spans="1:4" ht="15.75">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
@@ -739,7 +739,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="47.25">
+    <row r="9" spans="1:4" ht="15.75">
       <c r="A9" s="1" t="s">
         <v>31</v>
       </c>
@@ -753,7 +753,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="31.5">
+    <row r="10" spans="1:4" ht="15.75">
       <c r="A10" s="1" t="s">
         <v>35</v>
       </c>
@@ -767,7 +767,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="47.25">
+    <row r="11" spans="1:4" ht="15.75">
       <c r="A11" s="1" t="s">
         <v>39</v>
       </c>
@@ -781,7 +781,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="31.5">
+    <row r="12" spans="1:4" ht="15.75">
       <c r="A12" s="1" t="s">
         <v>43</v>
       </c>
@@ -795,7 +795,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="47.25">
+    <row r="13" spans="1:4" ht="15.75">
       <c r="A13" s="1" t="s">
         <v>47</v>
       </c>
@@ -809,7 +809,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="47.25">
+    <row r="14" spans="1:4" ht="31.5">
       <c r="A14" s="1" t="s">
         <v>51</v>
       </c>
@@ -823,7 +823,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="47.25">
+    <row r="15" spans="1:4" ht="15.75">
       <c r="A15" s="1" t="s">
         <v>55</v>
       </c>
@@ -837,7 +837,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="47.25">
+    <row r="16" spans="1:4" ht="15.75">
       <c r="A16" s="1" t="s">
         <v>59</v>
       </c>
@@ -851,7 +851,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="31.5">
+    <row r="17" spans="1:4" ht="15.75">
       <c r="A17" s="1" t="s">
         <v>63</v>
       </c>
@@ -865,7 +865,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="31.5">
+    <row r="18" spans="1:4" ht="15.75">
       <c r="A18" s="1" t="s">
         <v>67</v>
       </c>
@@ -879,7 +879,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="31.5">
+    <row r="19" spans="1:4" ht="15.75">
       <c r="A19" s="1" t="s">
         <v>71</v>
       </c>
@@ -893,7 +893,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="31.5">
+    <row r="20" spans="1:4" ht="15.75">
       <c r="A20" s="1" t="s">
         <v>75</v>
       </c>
@@ -907,7 +907,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="31.5">
+    <row r="21" spans="1:4" ht="15.75">
       <c r="A21" s="1" t="s">
         <v>79</v>
       </c>

</xml_diff>